<commit_message>
addedlogin for everyother method
</commit_message>
<xml_diff>
--- a/src/test/resources/LoginData.xlsx
+++ b/src/test/resources/LoginData.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2492331\Downloads\seleniumproject1\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B1636E9-206B-4343-B53A-7B66958EE863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2BC043-7D52-4444-89EE-889D5745E06B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{067AC5BB-FDC2-45E3-AC8D-8386880505A1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{067AC5BB-FDC2-45E3-AC8D-8386880505A1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="MoviegoerValid" sheetId="1" r:id="rId1"/>
+    <sheet name="MoviegoerInvalid" sheetId="2" r:id="rId2"/>
+    <sheet name="OwnerValid" sheetId="3" r:id="rId3"/>
+    <sheet name="OwnerInvalid" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
   <si>
     <t xml:space="preserve">username   </t>
   </si>
@@ -47,22 +50,31 @@
     <t>password</t>
   </si>
   <si>
-    <t>tomsmith</t>
-  </si>
-  <si>
-    <t>SuperSecretPassword!</t>
-  </si>
-  <si>
-    <t>wrongpassword</t>
-  </si>
-  <si>
-    <t>smith</t>
-  </si>
-  <si>
     <t>user1</t>
   </si>
   <si>
     <t>user1@g.com</t>
+  </si>
+  <si>
+    <t>expectedUrl</t>
+  </si>
+  <si>
+    <t>https://cinebookfrontend.netlify.app/movies</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>https://cinebookfrontend.netlify.app/login</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>tomsmith1</t>
+  </si>
+  <si>
+    <t>https://cinebookfrontend.netlify.app/manage-movies</t>
   </si>
 </sst>
 </file>
@@ -112,12 +124,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -457,7 +472,7 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -467,32 +482,25 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="1"/>
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
       <c r="C3" s="1"/>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
       <c r="C4" s="1"/>
     </row>
   </sheetData>
@@ -501,4 +509,114 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1E6CBC9-7382-4C02-B3A1-46B3C0491713}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="38.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <v>123</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD58142-B8A1-4B7F-92D9-C68D66064350}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.26953125" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" customWidth="1"/>
+    <col min="3" max="3" width="43.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{92A2B33B-C0D9-4A6F-AAE5-8DE139931CAB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45218F8C-066B-49AC-95A8-E8C30AB40C49}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="36.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>123</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>